<commit_message>
Just made some new prior files
</commit_message>
<xml_diff>
--- a/src/matlab/Matlab v.1.0/daugaard_standard.xlsx
+++ b/src/matlab/Matlab v.1.0/daugaard_standard.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <workbookPr/>
   <bookViews>
     <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Geology1" sheetId="2" r:id="rId3"/>
-    <sheet name="Geology2" sheetId="3" r:id="rId5"/>
-    <sheet name="Resistivity" sheetId="4" r:id="rId6"/>
+    <sheet name="Geology1" sheetId="1" r:id="rId2"/>
+    <sheet name="Geology2" sheetId="2" r:id="rId4"/>
+    <sheet name="Resistivity" sheetId="3" r:id="rId5"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="48" uniqueCount="36">
   <si>
     <t>Class</t>
   </si>
@@ -96,15 +95,9 @@
     <t>Probabilities</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>0.35,0.35,0.20,0.10</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>Min no of layers</t>
   </si>
   <si>
@@ -124,33 +117,6 @@
   </si>
   <si>
     <t>Min depth</t>
-  </si>
-  <si>
-    <t>Class</t>
-  </si>
-  <si>
-    <t>Organic rich</t>
-  </si>
-  <si>
-    <t>Meltwater sand</t>
-  </si>
-  <si>
-    <t>Till</t>
-  </si>
-  <si>
-    <t>Meltwater clay</t>
-  </si>
-  <si>
-    <t>Gravel</t>
-  </si>
-  <si>
-    <t>Miocene sand</t>
-  </si>
-  <si>
-    <t>Miocene clay</t>
-  </si>
-  <si>
-    <t>Paleogene clay</t>
   </si>
   <si>
     <t>Resistivity</t>
@@ -162,7 +128,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -200,8 +166,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -341,8 +307,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -365,25 +331,25 @@
         <v>25</v>
       </c>
       <c r="C1" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="F1" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="G1" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="H1" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="I1" s="0" t="s">
         <v>33</v>
-      </c>
-      <c r="H1" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="I1" s="0" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2">
@@ -391,7 +357,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C2" s="0">
         <v>1</v>
@@ -420,7 +386,7 @@
         <v>22</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C3" s="0">
         <v>2</v>
@@ -449,7 +415,7 @@
         <v>23</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C4" s="0">
         <v>2</v>
@@ -478,7 +444,7 @@
         <v>24</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C5" s="0">
         <v>1</v>
@@ -506,8 +472,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -518,18 +484,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="B2" s="0">
         <v>30</v>
@@ -540,7 +506,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="B3" s="0">
         <v>130</v>
@@ -551,7 +517,7 @@
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="B4" s="0">
         <v>50</v>
@@ -562,7 +528,7 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="B5" s="0">
         <v>20</v>
@@ -573,7 +539,7 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="B6" s="0">
         <v>200</v>
@@ -584,7 +550,7 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="B7" s="0">
         <v>110</v>
@@ -595,7 +561,7 @@
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>43</v>
+        <v>7</v>
       </c>
       <c r="B8" s="0">
         <v>25</v>
@@ -606,7 +572,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="B9" s="0">
         <v>5</v>

</xml_diff>